<commit_message>
Update CN/EN pages, add QR code images, update translations
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/prop/translation/core-products.xlsx
+++ b/prop/translation/core-products.xlsx
@@ -92,7 +92,7 @@
     <t>Force-Control Ready</t>
   </si>
   <si>
-    <t>原生力控</t>
+    <t>原生力控关节</t>
   </si>
   <si>
     <t>High Force Sensitivity</t>
@@ -200,7 +200,30 @@
     <t>Ultra-Lightweight / Humanoid</t>
   </si>
   <si>
-    <t>超轻量化 / 人形适配</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>超轻量化</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>仿人构型</t>
+    </r>
   </si>
   <si>
     <t>RM Series</t>
@@ -254,7 +277,7 @@
     <t>Humanoid</t>
   </si>
   <si>
-    <t>人形适配</t>
+    <t>仿人构型</t>
   </si>
   <si>
     <t>RX Series</t>
@@ -383,7 +406,7 @@
     <t>Advanced dexterous hands — engineered for human-like manipulation and seamless integration with the RealMan ecosystem.</t>
   </si>
   <si>
-    <t>先进灵巧手，专为拟人化操作精研，完美融入睿尔曼生态体系</t>
+    <t>先进灵巧手，专为拟人化操作研制，完美融入睿尔曼生态体系</t>
   </si>
 </sst>
 </file>
@@ -1642,7 +1665,7 @@
       <c r="A27" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="6" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1738,7 +1761,7 @@
       <c r="A39" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="6" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>